<commit_message>
Add miscellaneous modified parts - main part is power inlet for Ender3 switch assembly
</commit_message>
<xml_diff>
--- a/BOM_Trident170.xlsx
+++ b/BOM_Trident170.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/fc550a2baf076e0f/Documents/CAD Designs/3D Printers/Trender3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F452C2A-D417-4627-A525-8EC5946BF174}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="8_{8F452C2A-D417-4627-A525-8EC5946BF174}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CB88C5D0-8663-4C83-94DE-17DDDD62CBC6}"/>
   <bookViews>
-    <workbookView xWindow="585" yWindow="3300" windowWidth="28800" windowHeight="15345" xr2:uid="{84FBEF0A-233D-4E74-B7B4-DA8123BDCB49}"/>
+    <workbookView xWindow="4080" yWindow="2070" windowWidth="28800" windowHeight="15345" xr2:uid="{84FBEF0A-233D-4E74-B7B4-DA8123BDCB49}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="generated_bom" localSheetId="0">Sheet1!$A$1:$D$115</definedName>
+    <definedName name="generated_bom" localSheetId="0">Sheet1!$A$1:$D$117</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="147">
   <si>
     <t>Category</t>
   </si>
@@ -171,9 +171,6 @@
     <t>Linear Rail MGN12H 220mm</t>
   </si>
   <si>
-    <t>Linear Rail MGN9H 220mm</t>
-  </si>
-  <si>
     <t>GT2 Open Belt LL-2GT-6 (6mm wide) - 1370mm</t>
   </si>
   <si>
@@ -375,9 +372,6 @@
     <t>Misumi HFSB5-2020-290-TPW</t>
   </si>
   <si>
-    <t>Misumi HFSB5-2020-250-LTP</t>
-  </si>
-  <si>
     <t>Misumi HFSB5-2020-250</t>
   </si>
   <si>
@@ -426,27 +420,86 @@
     <t>Keenovo Silicone AC Heater w/ thermistor - 120x120mm (200W)</t>
   </si>
   <si>
-    <t>2040x420</t>
-  </si>
-  <si>
-    <t>4040x290 and 2020x290</t>
-  </si>
-  <si>
-    <t>2020x290</t>
-  </si>
-  <si>
-    <t>2020x152</t>
-  </si>
-  <si>
-    <t>2020x250</t>
+    <t>Linear Rail MGN9H 230mm</t>
+  </si>
+  <si>
+    <t>Can we fit a 230 here?</t>
+  </si>
+  <si>
+    <t>Y can be 230 with custom parts</t>
+  </si>
+  <si>
+    <t>Use leadscrews and coupler</t>
+  </si>
+  <si>
+    <t>2020x152 (bed 2)</t>
+  </si>
+  <si>
+    <t>2020x290 (bed 1)</t>
+  </si>
+  <si>
+    <t>4040x290 (lower back)</t>
+  </si>
+  <si>
+    <t>Misumi HFSB5-2020-260-LTP</t>
+  </si>
+  <si>
+    <t>2020x250 (X axis)</t>
+  </si>
+  <si>
+    <t>2020x160 (A/B connector back)</t>
+  </si>
+  <si>
+    <t>2020x290 (Y axis)</t>
+  </si>
+  <si>
+    <t>2040x400 (frame corners)</t>
+  </si>
+  <si>
+    <t>2040x330 (frame upper left/right)</t>
+  </si>
+  <si>
+    <t>TPW</t>
+  </si>
+  <si>
+    <t>Tapped both ends</t>
+  </si>
+  <si>
+    <t>LTP</t>
+  </si>
+  <si>
+    <t>Tapped one end</t>
+  </si>
+  <si>
+    <t>AH&lt;n&gt;</t>
+  </si>
+  <si>
+    <t>Access hole at position &lt;n&gt;</t>
+  </si>
+  <si>
+    <t>2020x260 (Z axis back)</t>
+  </si>
+  <si>
+    <t>4040x290 (frame lower front/sides)</t>
+  </si>
+  <si>
+    <t>180x180 Saladfork/Micron</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -474,8 +527,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -794,13 +848,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E043611C-4158-4461-A724-8FE30BC704BE}">
-  <dimension ref="A1:D115"/>
+  <dimension ref="A1:G117"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="58.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="4.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -1071,7 +1125,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
         <v>37</v>
       </c>
@@ -1079,7 +1133,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>38</v>
       </c>
@@ -1087,7 +1141,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
         <v>39</v>
       </c>
@@ -1095,7 +1149,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
         <v>40</v>
       </c>
@@ -1103,103 +1157,109 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
         <v>41</v>
       </c>
       <c r="C37">
         <v>1</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D37" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
-        <v>42</v>
+        <v>125</v>
       </c>
       <c r="C38">
         <v>5</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D38" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C39">
         <v>2</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>43</v>
+      </c>
+      <c r="B40" t="s">
         <v>44</v>
-      </c>
-      <c r="B40" t="s">
-        <v>45</v>
       </c>
       <c r="C40">
         <v>4</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>45</v>
+      </c>
+      <c r="B41" t="s">
         <v>46</v>
-      </c>
-      <c r="B41" t="s">
-        <v>47</v>
       </c>
       <c r="C41">
         <v>2</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C42">
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
+        <v>48</v>
+      </c>
+      <c r="C43">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B44" t="s">
         <v>49</v>
       </c>
-      <c r="C43">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B44" t="s">
+      <c r="C44">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B45" t="s">
         <v>50</v>
       </c>
-      <c r="C44">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B45" t="s">
+      <c r="C45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B46" t="s">
         <v>51</v>
       </c>
-      <c r="C45">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B46" t="s">
+      <c r="C46">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B47" t="s">
         <v>52</v>
       </c>
-      <c r="C46">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B47" t="s">
+      <c r="C47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B48" t="s">
         <v>53</v>
-      </c>
-      <c r="C47">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B48" t="s">
-        <v>54</v>
       </c>
       <c r="C48">
         <v>2</v>
@@ -1207,7 +1267,7 @@
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B49" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C49">
         <v>1</v>
@@ -1215,7 +1275,7 @@
     </row>
     <row r="50" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B50" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C50">
         <v>1</v>
@@ -1223,7 +1283,7 @@
     </row>
     <row r="51" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B51" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C51">
         <v>1</v>
@@ -1231,7 +1291,7 @@
     </row>
     <row r="52" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B52" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C52">
         <v>3</v>
@@ -1239,7 +1299,7 @@
     </row>
     <row r="53" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B53" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C53">
         <v>1</v>
@@ -1247,7 +1307,7 @@
     </row>
     <row r="54" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B54" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C54">
         <v>6</v>
@@ -1255,7 +1315,7 @@
     </row>
     <row r="55" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C55">
         <v>1</v>
@@ -1263,7 +1323,7 @@
     </row>
     <row r="56" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B56" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C56">
         <v>1</v>
@@ -1271,7 +1331,7 @@
     </row>
     <row r="57" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B57" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C57">
         <v>1</v>
@@ -1279,7 +1339,7 @@
     </row>
     <row r="58" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B58" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C58">
         <v>1</v>
@@ -1287,7 +1347,7 @@
     </row>
     <row r="59" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B59" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C59">
         <v>1</v>
@@ -1295,7 +1355,7 @@
     </row>
     <row r="60" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B60" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C60">
         <v>1</v>
@@ -1303,7 +1363,7 @@
     </row>
     <row r="61" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B61" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C61">
         <v>1</v>
@@ -1311,7 +1371,7 @@
     </row>
     <row r="62" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B62" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C62">
         <v>1</v>
@@ -1319,7 +1379,7 @@
     </row>
     <row r="63" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B63" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C63">
         <v>1</v>
@@ -1327,141 +1387,144 @@
     </row>
     <row r="64" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B64" t="s">
+        <v>69</v>
+      </c>
+      <c r="C64">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B65" t="s">
         <v>70</v>
-      </c>
-      <c r="C64">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B65" t="s">
-        <v>71</v>
       </c>
       <c r="C65">
         <v>3</v>
       </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D65" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
+        <v>71</v>
+      </c>
+      <c r="B66" t="s">
         <v>72</v>
       </c>
-      <c r="B66" t="s">
+      <c r="C66">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B67" t="s">
         <v>73</v>
       </c>
-      <c r="C66">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B67" t="s">
+      <c r="C67">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B68" t="s">
         <v>74</v>
       </c>
-      <c r="C67">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B68" t="s">
+      <c r="C68">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B69" t="s">
         <v>75</v>
       </c>
-      <c r="C68">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B69" t="s">
+      <c r="C69">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B70" t="s">
         <v>76</v>
-      </c>
-      <c r="C69">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B70" t="s">
-        <v>77</v>
       </c>
       <c r="C70">
         <v>6</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B71" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C71">
         <v>3</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B72" t="s">
+        <v>78</v>
+      </c>
+      <c r="C72">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B73" t="s">
         <v>79</v>
       </c>
-      <c r="C72">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B73" t="s">
+      <c r="C73">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B74" t="s">
         <v>80</v>
       </c>
-      <c r="C73">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B74" t="s">
+      <c r="C74">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B75" t="s">
         <v>81</v>
-      </c>
-      <c r="C74">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B75" t="s">
-        <v>82</v>
       </c>
       <c r="C75">
         <v>8</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B76" t="s">
+        <v>82</v>
+      </c>
+      <c r="C76">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
         <v>83</v>
       </c>
-      <c r="C76">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
+      <c r="B77" t="s">
         <v>84</v>
-      </c>
-      <c r="B77" t="s">
-        <v>85</v>
       </c>
       <c r="C77">
         <v>40</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B78" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C78">
         <v>5</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B79" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C79">
         <v>10</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B80" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C80">
         <v>10</v>
@@ -1469,7 +1532,7 @@
     </row>
     <row r="81" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B81" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C81">
         <v>100</v>
@@ -1477,7 +1540,7 @@
     </row>
     <row r="82" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B82" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C82">
         <v>10</v>
@@ -1485,7 +1548,7 @@
     </row>
     <row r="83" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B83" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C83">
         <v>5</v>
@@ -1493,7 +1556,7 @@
     </row>
     <row r="84" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B84" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C84">
         <v>4</v>
@@ -1501,7 +1564,7 @@
     </row>
     <row r="85" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B85" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C85">
         <v>2</v>
@@ -1509,7 +1572,7 @@
     </row>
     <row r="86" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B86" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C86">
         <v>40</v>
@@ -1517,7 +1580,7 @@
     </row>
     <row r="87" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B87" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C87">
         <v>2</v>
@@ -1525,7 +1588,7 @@
     </row>
     <row r="88" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B88" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C88">
         <v>1</v>
@@ -1533,7 +1596,7 @@
     </row>
     <row r="89" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B89" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C89">
         <v>5</v>
@@ -1541,7 +1604,7 @@
     </row>
     <row r="90" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B90" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C90">
         <v>2</v>
@@ -1549,7 +1612,7 @@
     </row>
     <row r="91" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B91" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C91">
         <v>1</v>
@@ -1557,7 +1620,7 @@
     </row>
     <row r="92" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B92" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C92">
         <v>5</v>
@@ -1565,7 +1628,7 @@
     </row>
     <row r="93" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B93" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C93">
         <v>40</v>
@@ -1573,7 +1636,7 @@
     </row>
     <row r="94" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B94" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C94">
         <v>40</v>
@@ -1581,7 +1644,7 @@
     </row>
     <row r="95" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B95" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C95">
         <v>1</v>
@@ -1589,62 +1652,83 @@
     </row>
     <row r="96" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B96" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C96">
         <v>3</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B97" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C97">
         <v>3</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
+        <v>105</v>
+      </c>
+      <c r="B98" t="s">
         <v>106</v>
-      </c>
-      <c r="B98" t="s">
-        <v>107</v>
       </c>
       <c r="C98">
         <v>2</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B99" t="s">
+        <v>110</v>
+      </c>
+      <c r="C99">
+        <v>4</v>
+      </c>
+      <c r="D99" t="s">
+        <v>136</v>
+      </c>
+      <c r="F99" t="s">
+        <v>138</v>
+      </c>
+      <c r="G99" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B100" t="s">
         <v>108</v>
       </c>
-      <c r="C99">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B100" t="s">
-        <v>109</v>
-      </c>
       <c r="C100">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D100" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+      <c r="F100" t="s">
+        <v>140</v>
+      </c>
+      <c r="G100" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B101" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C101">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D101" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+      <c r="F101" t="s">
+        <v>142</v>
+      </c>
+      <c r="G101" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B102" t="s">
         <v>111</v>
       </c>
@@ -1655,125 +1739,150 @@
         <v>131</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B103" t="s">
+        <v>108</v>
+      </c>
+      <c r="C103">
+        <v>2</v>
+      </c>
+      <c r="D103" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B104" t="s">
+        <v>109</v>
+      </c>
+      <c r="C104">
+        <v>1</v>
+      </c>
+      <c r="D104" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B105" t="s">
+        <v>132</v>
+      </c>
+      <c r="C105">
+        <v>1</v>
+      </c>
+      <c r="D105" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B106" t="s">
+        <v>107</v>
+      </c>
+      <c r="C106">
+        <v>1</v>
+      </c>
+      <c r="D106" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B107" t="s">
+        <v>113</v>
+      </c>
+      <c r="C107">
+        <v>1</v>
+      </c>
+      <c r="D107" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B108" t="s">
         <v>112</v>
       </c>
-      <c r="C103">
-        <v>4</v>
-      </c>
-      <c r="D103" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B104" t="s">
-        <v>113</v>
-      </c>
-      <c r="C104">
-        <v>1</v>
-      </c>
-      <c r="D104" t="s">
+      <c r="C108">
+        <v>1</v>
+      </c>
+      <c r="D108" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B105" t="s">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
         <v>114</v>
       </c>
-      <c r="C105">
-        <v>1</v>
-      </c>
-      <c r="D105" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B106" t="s">
+      <c r="B109" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="C106">
-        <v>1</v>
-      </c>
-      <c r="D106" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A107" t="s">
-        <v>116</v>
-      </c>
-      <c r="B107" t="s">
-        <v>117</v>
-      </c>
-      <c r="C107">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B108" t="s">
-        <v>118</v>
-      </c>
-      <c r="C108">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B109" t="s">
-        <v>119</v>
       </c>
       <c r="C109">
         <v>2</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B110" t="s">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B110" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C110">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B111" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C111">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B112" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C112">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B113" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C113">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
         <v>120</v>
       </c>
-      <c r="C110">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B111" t="s">
+      <c r="B114" t="s">
         <v>121</v>
       </c>
-      <c r="C111">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A112" t="s">
+      <c r="C114">
+        <v>1</v>
+      </c>
+      <c r="D114" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B115" t="s">
         <v>122</v>
       </c>
-      <c r="B112" t="s">
+      <c r="C115">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B116" t="s">
         <v>123</v>
       </c>
-      <c r="C112">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="113" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B113" t="s">
+      <c r="C116">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B117" t="s">
         <v>124</v>
       </c>
-      <c r="C113">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="114" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B114" t="s">
-        <v>125</v>
-      </c>
-      <c r="C114">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="115" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B115" t="s">
-        <v>126</v>
-      </c>
-      <c r="C115">
+      <c r="C117">
         <v>1</v>
       </c>
     </row>

</xml_diff>